<commit_message>
Add experiment outputs and notebook updates
Update notebooks to use the new INDEX_CSV and output directory (execution counts bumped and save path adjusted). Add generated notebook outputs (confusion matrices, row-normalized matrix, per-class metrics) and many FinalReport evidence images/JSON/Excel artifacts. Also include minor Prototype4 frontend/index.html and SystemTests.xlsx updates.
</commit_message>
<xml_diff>
--- a/Prototype4/testing/SystemTests.xlsx
+++ b/Prototype4/testing/SystemTests.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cianan/Documents/College/GitHub/FYP/Prototype3/testing/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/cianan/Documents/College/GitHub/FYP/Prototype4/testing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{104790FC-7F7D-5B4D-B7EB-54E4945AF206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52C6CCAD-0843-F643-9D98-4710ADA43335}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="24000" xr2:uid="{2F330C29-766A-3B4B-9059-8C837B743AAD}"/>
+    <workbookView xWindow="38400" yWindow="1340" windowWidth="38400" windowHeight="23520" xr2:uid="{2F330C29-766A-3B4B-9059-8C837B743AAD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="91">
   <si>
     <t>TestID</t>
   </si>
@@ -106,9 +106,6 @@
 .Status message updates to selected model</t>
   </si>
   <si>
-    <t>Upload valid WAV file and predict</t>
-  </si>
-  <si>
     <t>ST-03</t>
   </si>
   <si>
@@ -128,9 +125,6 @@
   </si>
   <si>
     <t>Verify end-to-end prediction using uploaded audio.</t>
-  </si>
-  <si>
-    <t>Known-good WAV test file of at least 10 seconds available.</t>
   </si>
   <si>
     <t>1.Open the frontend
@@ -146,21 +140,10 @@
 .No frontend or backend error occurs</t>
   </si>
   <si>
-    <t>Record audio over 10 seconds and predict</t>
-  </si>
-  <si>
     <t>Verify end-to-end prediction using browser microphone recording.</t>
   </si>
   <si>
     <t>Working microphone permission granted.</t>
-  </si>
-  <si>
-    <t>1.Open the frontend
-2.Select a model
-3.Click Start Recording
-4.Speak for at least 10 seconds
-5.Click Stop Recording
-6.Click Predict Accent</t>
   </si>
   <si>
     <t>.Recording countdown works correctly
@@ -201,11 +184,6 @@
 3.Click Predict Accent</t>
   </si>
   <si>
-    <t>.System does not attempt prediction
-.User receives clear message such as “No model selected.”
-.No crash occurs</t>
-  </si>
-  <si>
     <t>ST-09</t>
   </si>
   <si>
@@ -303,9 +281,88 @@
 5.Run prediction again</t>
   </si>
   <si>
-    <t>.Frontend loads updated model list without code changes
-.Prediction still works through same UI
-.Confirms modular architecture</t>
+    <t>Record audio predict</t>
+  </si>
+  <si>
+    <t>1.Open the frontend
+2.Select a model
+3.Click Start Recording
+4.Speak for at least 10 seconds
+5.Recording auto-stops
+6.Click Predict Accent</t>
+  </si>
+  <si>
+    <t>.System does not attempt prediction
+.Predict button remains grey/ unclickable.
+.No crash occurs</t>
+  </si>
+  <si>
+    <t>Main frontend loads successfully with no issues. Swagger docs load succesfully. No errors</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Actual model names replaces loading models, a default is selcted, status message updates to say which is selcted</t>
+  </si>
+  <si>
+    <t>Known good  test file of at least 10 seconds available for each file type.</t>
+  </si>
+  <si>
+    <t>Upload valid AAC, AIFF, ALAC, AMR, OGG, WMA, WAV,FLAC,MP3,M4A, WebM file and predict</t>
+  </si>
+  <si>
+    <t>pass: aiff,  flac, aac, m4a, mp3, ogg, webm, amr FAILED: wma</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Pass, with exception</t>
+  </si>
+  <si>
+    <t>For report</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Differences in prediction outputs across formats (e.g., AMR) suggest that encoding and compression may influence feature extraction and model performance.. Support for a wide range of audio formats was achieved through backend decoding. However, WMA files were not successfully processed, highlighting a limitation in format compatibility. </t>
+  </si>
+  <si>
+    <t>Had major issue, managed to fix</t>
+  </si>
+  <si>
+    <t>Recording countdown works. Predict button becomes available after. Playback oreview is shown. Prediction appears on map. Map updates correctly</t>
+  </si>
+  <si>
+    <t>I think wma not passing is acceptable on frontend. Worked using api. Interseting amr file gave differentresult</t>
+  </si>
+  <si>
+    <t>Had a minor issue of prediction text not showing. It was just a colour issue quickly resovled.</t>
+  </si>
+  <si>
+    <t>Recordings shorter than 10 seconds were correctly rejected. The predict button remained disabled, and the system displayed a clear message indicating the minimum recording requirement.</t>
+  </si>
+  <si>
+    <t>The frontend enforces model selection by automatically selecting a default model when available, preventing the user from initiating prediction without a valid model. Direct API testing without a model resulted in an appropriate HTTP error response.</t>
+  </si>
+  <si>
+    <t>Recording of non-speech or invalid audio input did not cause system failure. The backend processed the input and returned a prediction, though results were not meaningful. The system remained stable throughout.</t>
+  </si>
+  <si>
+    <t>The frontend restricted file selection to supported audio formats. When bypassed via API testing (e.g., uploading a .jpg file), the backend returned a clear error message without crashing.</t>
+  </si>
+  <si>
+    <t>The prediction panel correctly displayed the selected model, predicted label, confidence value, and probability distribution. A minor UI issue with text visibility was identified and resolved.</t>
+  </si>
+  <si>
+    <t>The map correctly highlighted the predicted province, cleared any previous highlights, and matched the prediction output displayed in the interface.</t>
+  </si>
+  <si>
+    <t>After disabling the dummy backend plugin, the models returned by /api/models changed accordingly, and the frontend dropdown updated after page reload without any frontend code changes. Prediction continued to work successfully with the remaining models, and the map updated correctly.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	•	frontend updated after reload
+	•	no frontend code changes required
+	•	prediction still worked</t>
   </si>
 </sst>
 </file>
@@ -347,16 +404,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="10">
+  <dxfs count="12">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -401,9 +465,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6C67DC76-66FB-9146-BD7D-31416DAFF067}" name="Table1" displayName="Table1" ref="A1:H12" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0">
-  <autoFilter ref="A1:H12" xr:uid="{6C67DC76-66FB-9146-BD7D-31416DAFF067}"/>
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6C67DC76-66FB-9146-BD7D-31416DAFF067}" name="Table1" displayName="Table1" ref="A1:J12" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J12" xr:uid="{6C67DC76-66FB-9146-BD7D-31416DAFF067}"/>
+  <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{DD7121A9-17D7-1D44-89B9-109712E4B970}" name="TestID" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{FAD7E897-7E06-9947-AAF4-44B5BFB912FF}" name="TestName" dataDxfId="8"/>
     <tableColumn id="3" xr3:uid="{B6213037-1096-754F-BD7D-4595E2502D4E}" name="Objective" dataDxfId="7"/>
@@ -412,6 +476,8 @@
     <tableColumn id="6" xr3:uid="{2AC907FF-628B-3049-95BC-A677C9C0BD86}" name="ExpectedResults" dataDxfId="4"/>
     <tableColumn id="7" xr3:uid="{ACC8188B-6AF4-7342-9E85-2DE5573DB019}" name="ActualResult" dataDxfId="3"/>
     <tableColumn id="8" xr3:uid="{0EA3886C-4C11-7A44-A85D-A84B809F648E}" name="Pass/Fail" dataDxfId="2"/>
+    <tableColumn id="9" xr3:uid="{6813877C-98A2-C84B-B706-F0F776F6FF42}" name="Notes" dataDxfId="1"/>
+    <tableColumn id="10" xr3:uid="{2C57DD04-1375-5942-936E-03D361273F87}" name="For report" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -734,7 +800,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6231815A-A563-5541-A681-F72F0F749DB7}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.83203125" style="1" customWidth="1"/>
@@ -742,10 +808,13 @@
     <col min="3" max="4" width="27" style="1" customWidth="1"/>
     <col min="5" max="5" width="41.5" style="1" customWidth="1"/>
     <col min="6" max="6" width="48" style="1" customWidth="1"/>
-    <col min="7" max="8" width="15.83203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="26.33203125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="22.1640625" customWidth="1"/>
+    <col min="10" max="10" width="28.6640625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -770,8 +839,14 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>77</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" ht="68" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="68" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -790,8 +865,15 @@
       <c r="F2" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="G2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="I2" s="1"/>
     </row>
-    <row r="3" spans="1:8" ht="51" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="68" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
@@ -810,186 +892,264 @@
       <c r="F3" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="G3" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="I3" s="1"/>
     </row>
-    <row r="4" spans="1:8" ht="85" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ht="85" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="102" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E4" s="1" t="s">
+      <c r="B5" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>30</v>
       </c>
+      <c r="E5" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="I5" s="1"/>
+      <c r="J5" s="2" t="s">
+        <v>79</v>
+      </c>
     </row>
-    <row r="5" spans="1:8" ht="100" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
+    <row r="6" spans="1:10" ht="136" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="D6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>35</v>
       </c>
+      <c r="G6" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="I6" s="1"/>
     </row>
-    <row r="6" spans="1:8" ht="69" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+    <row r="7" spans="1:10" ht="153" x14ac:dyDescent="0.2">
+      <c r="A7" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E6" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="E7" s="1" t="s">
         <v>39</v>
       </c>
+      <c r="F7" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="I7" s="1"/>
     </row>
-    <row r="7" spans="1:8" ht="53" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
+    <row r="8" spans="1:10" ht="136" x14ac:dyDescent="0.2">
+      <c r="A8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B8" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="I8" s="1"/>
+    </row>
+    <row r="9" spans="1:10" ht="119" x14ac:dyDescent="0.2">
+      <c r="A9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="I9" s="1"/>
+    </row>
+    <row r="10" spans="1:10" ht="119" x14ac:dyDescent="0.2">
+      <c r="A10" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="B10" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="I10" s="1"/>
+      <c r="J10" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="102" x14ac:dyDescent="0.2">
+      <c r="A11" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>44</v>
-      </c>
+      <c r="B11" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="I11" s="1"/>
     </row>
-    <row r="8" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="68" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="51" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B11" s="1" t="s">
+    <row r="12" spans="1:10" ht="187" x14ac:dyDescent="0.2">
+      <c r="A12" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="B12" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="C12" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="D12" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" ht="102" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="H12" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>71</v>
-      </c>
+      <c r="I12" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>